<commit_message>
Expand question bank to 214 and apply UI/content fixes
- Grow data/questions.xlsx from 45 to 214 questions across 11 categories
  (adds This or That, Family, What Grounds You, Your Posse; city-targeted
  prompts for Chicago/NYC/LA/DC). Depth mix ~39/32/21/8 (warm-up heavy).
- Remove all emojis from the UI; category tags are now clean color-coded
  text (small color dot on chips, color swatch on browse headers).
- Expand category palette to 12 WCAG-AA colors (white text >= 4.5:1).
- Add fine-print footer disclaimer (independent project + contact) and a
  "Skipping any question is always okay" reassurance line.
- Broaden .gitignore to exclude all of data/wnrs/ (local source only).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/questions.xlsx
+++ b/data/questions.xlsx
@@ -425,12 +425,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C46"/>
+  <dimension ref="A1:C215"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="72" customWidth="1" min="3" max="3"/>
+    <col width="82" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -558,517 +558,517 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Getting to Know You</t>
+          <t>Icebreakers</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>What are you most looking forward to about starting college?</t>
+          <t>What's the last thing that made you laugh out loud?</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Getting to Know You</t>
+          <t>Icebreakers</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>What's a class or subject you're secretly excited to take?</t>
+          <t>What's your go-to karaoke song?</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Getting to Know You</t>
+          <t>Icebreakers</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Who's someone you really look up to?</t>
+          <t>What are you looking forward to this week?</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Getting to Know You</t>
+          <t>Icebreakers</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>What's something you're really good at that people wouldn't guess?</t>
+          <t>What's the best thing you've eaten recently?</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Getting to Know You</t>
+          <t>Icebreakers</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>What did a typical weekend look like for you back home?</t>
+          <t>If today had a theme song, what would it be?</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Getting to Know You</t>
+          <t>Icebreakers</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>What's a movie or show you could rewatch a hundred times?</t>
+          <t>What's your comfort show — the one you rewatch on autopilot?</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Getting to Know You</t>
+          <t>Icebreakers</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>What's one thing on your bucket list for the next four years?</t>
+          <t>What's a snack you could eat every single day?</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Roots &amp; Cities</t>
+          <t>Icebreakers</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>What's the best food your city is known for?</t>
+          <t>What's on your phone wallpaper right now, and why?</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Roots &amp; Cities</t>
+          <t>Icebreakers</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>What's a spot in your hometown you'd take a friend to first?</t>
+          <t>What's your ideal way to spend a slow Sunday?</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Roots &amp; Cities</t>
+          <t>Icebreakers</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>What's something people get wrong about where you're from?</t>
+          <t>What's a small win you had recently?</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Roots &amp; Cities</t>
+          <t>Icebreakers</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>What will you miss most about home?</t>
+          <t>What's your usual order at a coffee shop or drive-thru?</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Roots &amp; Cities</t>
+          <t>Icebreakers</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>What's a word or phrase people say in your city that others don't?</t>
+          <t>What's something you're weirdly good at?</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Roots &amp; Cities</t>
+          <t>Icebreakers</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>What's a hidden gem in your neighborhood?</t>
+          <t>What three words would your closest friends use to describe you?</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Values &amp; Identity</t>
+          <t>Icebreakers</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>What's a value your family passed down that you carry with you?</t>
+          <t>What's a show everyone loves that you just never got into?</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Values &amp; Identity</t>
+          <t>Icebreakers</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>When do you feel most like yourself?</t>
+          <t>What's the last thing you got genuinely excited about?</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Values &amp; Identity</t>
+          <t>Getting to Know You</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>What's something you've changed your mind about recently?</t>
+          <t>What are you most looking forward to about starting college?</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Values &amp; Identity</t>
+          <t>Getting to Know You</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>What does "community" mean to you?</t>
+          <t>What's a class or subject you're secretly excited to take?</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Values &amp; Identity</t>
+          <t>Getting to Know You</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Who has shaped the way you see the world the most?</t>
+          <t>What's something you're really good at that people wouldn't guess?</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Values &amp; Identity</t>
+          <t>Getting to Know You</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>What's a part of your identity you're proud of?</t>
+          <t>What did a typical weekend look like for you back home?</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Dreams &amp; Goals</t>
+          <t>Getting to Know You</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>What made you say yes to Posse and to UW–Madison?</t>
+          <t>What's one thing on your bucket list for the next four years?</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Dreams &amp; Goals</t>
+          <t>Getting to Know You</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Where do you hope to be in ten years — big picture, no wrong answers?</t>
+          <t>What's your major, or best guess right now — and what pulled you toward it?</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Dreams &amp; Goals</t>
+          <t>Getting to Know You</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>What's something you want to be brave enough to try in college?</t>
+          <t>What did you want to be when you were little?</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Dreams &amp; Goals</t>
+          <t>Getting to Know You</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>What kind of impact do you want to have someday?</t>
+          <t>What have you been really into lately — a show, a hobby, a rabbit hole?</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Dreams &amp; Goals</t>
+          <t>Getting to Know You</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>What would "making the most of this" look like for you?</t>
+          <t>Are you more of a planner or a go-with-the-flow person?</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Dreams &amp; Goals</t>
+          <t>Getting to Know You</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>What's a goal you've never said out loud before?</t>
+          <t>What's a subject you didn't expect to love but did?</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Deeper Cuts</t>
+          <t>Getting to Know You</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>What's something you're nervous about that you don't say out loud much?</t>
+          <t>How do you recharge after a long week — around people or on your own?</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Deeper Cuts</t>
+          <t>Getting to Know You</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>What's a challenge you've come through that shaped who you are?</t>
+          <t>What's a skill you'd love to pick up during college?</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Deeper Cuts</t>
+          <t>Getting to Know You</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>What does "home" feel like to you, beyond a place?</t>
+          <t>When you're out with friends, what's your role — planner, driver, hype person, always-late one?</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Deeper Cuts</t>
+          <t>Getting to Know You</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>When was a time you felt truly supported by a group?</t>
+          <t>What's something from this past year you're proud of?</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Deeper Cuts</t>
+          <t>Getting to Know You</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>What's something you're still figuring out about yourself?</t>
+          <t>Who's someone you look up to, and what do you admire about them?</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Deeper Cuts</t>
+          <t>Getting to Know You</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>What do you hope your Posse remembers about you?</t>
+          <t>What's a place in Madison or on campus you're excited to explore?</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Just for Fun</t>
+          <t>Getting to Know You</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Would you rather be able to fly or be invisible?</t>
+          <t>What's a personal goal you're bringing into freshman year?</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Just for Fun</t>
+          <t>Getting to Know You</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Pineapple on pizza: yes or no? Defend your answer.</t>
+          <t>What do people usually get wrong about you when they first meet you?</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Just for Fun</t>
+          <t>Getting to Know You</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>What's the most useless talent you have?</t>
+          <t>What's your comfort meal when you're missing home?</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Just for Fun</t>
+          <t>Getting to Know You</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1076,52 +1076,2587 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>If you had to eat one meal for the rest of your life, what is it?</t>
+          <t>What's a hobby you had as a kid that you kind of miss?</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Just for Fun</t>
+          <t>Roots &amp; Cities</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Beach day or mountain day?</t>
+          <t>What's the best food your city is known for?</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Just for Fun</t>
+          <t>Roots &amp; Cities</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>What's your most controversial (totally non-serious) opinion?</t>
+          <t>What's a spot in your hometown you'd take a friend to first?</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
+          <t>Roots &amp; Cities</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>2</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>What's something people get wrong about where you're from?</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Roots &amp; Cities</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>2</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>What will you miss most about home?</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Roots &amp; Cities</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>2</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>What's a word or phrase people say in your city that others don't?</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Roots &amp; Cities</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>2</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>What's a hidden gem in your neighborhood?</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Roots &amp; Cities</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>1</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>If I visited your city for one day, what's the one thing you'd make me do?</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Roots &amp; Cities</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>2</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>What's a sound or a smell that instantly means home to you?</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Roots &amp; Cities</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>1</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Describe your neighborhood in three words.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Roots &amp; Cities</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>What's your city's unofficial rule that only locals know?</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Roots &amp; Cities</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>2</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>What's the skyline or view that makes you proud of where you're from?</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Roots &amp; Cities</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>3</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>What's something about your city you didn't appreciate until you were about to leave?</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Roots &amp; Cities</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>1</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>What's a tradition or yearly event your city does that you love?</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Roots &amp; Cities</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>2</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>What's a stereotype about your city that's actually kind of true — and one that's totally wrong?</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Roots &amp; Cities</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>3</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>How does where you grew up show up in who you are?</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Roots &amp; Cities</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>2</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>What's a place back home you already know you'll be homesick for?</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Roots &amp; Cities</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>1</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>What's a slang word from your city you're going to accidentally confuse people with here?</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Roots &amp; Cities</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>1</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>What does your city do better than anywhere else?</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Roots &amp; Cities</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>1</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Chicago crew — deep dish or tavern-style, and defend your answer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Roots &amp; Cities</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>2</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Chicago folks — what neighborhood are you repping, and what's it known for?</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Roots &amp; Cities</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>2</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Chicago people — what's the Chicago that tourists downtown never see?</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Roots &amp; Cities</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>1</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Chicago scholars — what's one thing about your city you'd defend to anyone?</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Roots &amp; Cities</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>2</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>NYC crew — which borough shaped you, and how?</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Roots &amp; Cities</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>1</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>New York folks — best slice spot near you, no debate?</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Roots &amp; Cities</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>2</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>NYC people — what's a New York habit you do without even noticing?</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Roots &amp; Cities</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>2</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>New York scholars — is the city's energy something you feed off of or need a break from?</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Roots &amp; Cities</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>2</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>LA crew — what's the LA that outsiders never get to see?</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Roots &amp; Cities</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>1</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>LA folks — beaches, mountains, or the city itself: what's your LA?</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Roots &amp; Cities</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>1</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>LA people — what's a spot or a food that says home to you?</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Roots &amp; Cities</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>2</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>LA scholars — what do people always get wrong about LA?</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Roots &amp; Cities</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>3</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>DC crew — is DC home, or just where you're from?</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Roots &amp; Cities</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>1</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>DC folks — go-to mumbo sauce order, or what's the DC food people sleep on?</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Roots &amp; Cities</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>2</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>DC people — what's the DC that has nothing to do with politics or monuments?</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Roots &amp; Cities</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>2</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>DC scholars — what neighborhood or quadrant are you from, and what's it like?</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Values &amp; Identity</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>3</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>What's a value your family passed down that you carry with you?</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Values &amp; Identity</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>3</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>When do you feel most like yourself?</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Values &amp; Identity</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>3</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>What's something you've changed your mind about recently?</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Values &amp; Identity</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>3</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>What does “community” mean to you?</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Values &amp; Identity</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>3</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Who has shaped the way you see the world the most?</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Values &amp; Identity</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>2</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>What's a part of your identity you're proud of?</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Values &amp; Identity</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>2</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>What's a cause or issue you genuinely care about?</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Values &amp; Identity</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>2</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>What's an unpopular opinion you'll stand behind?</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Values &amp; Identity</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>3</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>What's something you believed a few years ago that you see differently now?</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Values &amp; Identity</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>2</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>What's a green flag you look for in people?</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Values &amp; Identity</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>3</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>What's a value you refuse to compromise on?</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Values &amp; Identity</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>2</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>What's a part of your culture or background you're proud to carry?</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Values &amp; Identity</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>3</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>What's something people misunderstand about a community you belong to?</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Values &amp; Identity</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>2</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>When have you felt most proud to be you?</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Values &amp; Identity</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>4</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>What does integrity look like to you in everyday life?</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Values &amp; Identity</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>2</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>What's a quote, lyric, or saying you low-key live by?</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Dreams &amp; Goals</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>3</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>What made you say yes to Posse and to UW–Madison?</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Dreams &amp; Goals</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>3</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Where do you hope to be in ten years — big picture, no wrong answers?</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Dreams &amp; Goals</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>3</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>What's something you want to be brave enough to try in college?</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Dreams &amp; Goals</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>4</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>What kind of impact do you want to have someday?</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Dreams &amp; Goals</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>3</v>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>What would making the most of this look like for you?</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Dreams &amp; Goals</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>3</v>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>What's a goal you've never said out loud before?</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Dreams &amp; Goals</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>2</v>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>If money weren't a factor, what would you spend your life doing?</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Dreams &amp; Goals</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>3</v>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>What does success look like for you — on your own terms, not anyone else's?</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Dreams &amp; Goals</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>2</v>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Who's someone doing work you admire, and what draws you to it?</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Dreams &amp; Goals</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>4</v>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>What kind of person do you want to be by the time you graduate?</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Dreams &amp; Goals</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>4</v>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>What's a dream that feels a little too big to say out loud — but here goes?</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Dreams &amp; Goals</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>2</v>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>What's something you want to be known for?</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Dreams &amp; Goals</t>
+        </is>
+      </c>
+      <c r="B106" t="n">
+        <v>2</v>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>What's a skill or field you're excited to go deep on?</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Dreams &amp; Goals</t>
+        </is>
+      </c>
+      <c r="B107" t="n">
+        <v>3</v>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>If you could solve one problem in the world, what would you pick?</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Dreams &amp; Goals</t>
+        </is>
+      </c>
+      <c r="B108" t="n">
+        <v>2</v>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>What's a goal for this year — something you can actually start on soon?</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Dreams &amp; Goals</t>
+        </is>
+      </c>
+      <c r="B109" t="n">
+        <v>3</v>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>What would your younger self be amazed to see you doing now?</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Dreams &amp; Goals</t>
+        </is>
+      </c>
+      <c r="B110" t="n">
+        <v>4</v>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>What's a risk you hope you're brave enough to take?</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Dreams &amp; Goals</t>
+        </is>
+      </c>
+      <c r="B111" t="n">
+        <v>4</v>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>What does a life well spent mean to you?</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Dreams &amp; Goals</t>
+        </is>
+      </c>
+      <c r="B112" t="n">
+        <v>2</v>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Who do you want to make proud, and why?</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Dreams &amp; Goals</t>
+        </is>
+      </c>
+      <c r="B113" t="n">
+        <v>4</v>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>What legacy do you want to leave at UW — or anywhere?</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Deeper Cuts</t>
+        </is>
+      </c>
+      <c r="B114" t="n">
+        <v>4</v>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>What's something you're a little nervous about that you don't say out loud much?</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Deeper Cuts</t>
+        </is>
+      </c>
+      <c r="B115" t="n">
+        <v>3</v>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>What's a challenge you're proud of getting through?</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Deeper Cuts</t>
+        </is>
+      </c>
+      <c r="B116" t="n">
+        <v>3</v>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>What does home feel like to you, beyond a place?</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Deeper Cuts</t>
+        </is>
+      </c>
+      <c r="B117" t="n">
+        <v>3</v>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>When was a time you felt truly supported by a group?</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Deeper Cuts</t>
+        </is>
+      </c>
+      <c r="B118" t="n">
+        <v>3</v>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>What's something you're still figuring out about yourself?</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Deeper Cuts</t>
+        </is>
+      </c>
+      <c r="B119" t="n">
+        <v>4</v>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>How are you, really — the honest version?</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Deeper Cuts</t>
+        </is>
+      </c>
+      <c r="B120" t="n">
+        <v>3</v>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>What's a compliment that has always stuck with you?</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Deeper Cuts</t>
+        </is>
+      </c>
+      <c r="B121" t="n">
+        <v>4</v>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>What's a fear you're slowly getting better at facing?</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Deeper Cuts</t>
+        </is>
+      </c>
+      <c r="B122" t="n">
+        <v>3</v>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>What would you tell your younger self if you could?</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Deeper Cuts</t>
+        </is>
+      </c>
+      <c r="B123" t="n">
+        <v>3</v>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>What's a lesson that took you a long time to learn?</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Deeper Cuts</t>
+        </is>
+      </c>
+      <c r="B124" t="n">
+        <v>3</v>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>What's something you're hoping college helps you figure out?</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Deeper Cuts</t>
+        </is>
+      </c>
+      <c r="B125" t="n">
+        <v>3</v>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>What title would you give this chapter of your life?</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Deeper Cuts</t>
+        </is>
+      </c>
+      <c r="B126" t="n">
+        <v>3</v>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>When did you last surprise yourself?</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Deeper Cuts</t>
+        </is>
+      </c>
+      <c r="B127" t="n">
+        <v>4</v>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>What's a part of yourself you've fully made peace with?</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Deeper Cuts</t>
+        </is>
+      </c>
+      <c r="B128" t="n">
+        <v>4</v>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>What's something true about you that takes people a while to see?</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Deeper Cuts</t>
+        </is>
+      </c>
+      <c r="B129" t="n">
+        <v>4</v>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>What do you need more of in your life right now?</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
           <t>Just for Fun</t>
         </is>
       </c>
-      <c r="B46" t="n">
-        <v>1</v>
-      </c>
-      <c r="C46" t="inlineStr">
+      <c r="B130" t="n">
+        <v>1</v>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Would you rather be able to fly or be invisible?</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Just for Fun</t>
+        </is>
+      </c>
+      <c r="B131" t="n">
+        <v>1</v>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Pineapple on pizza: yes or no? Defend your answer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Just for Fun</t>
+        </is>
+      </c>
+      <c r="B132" t="n">
+        <v>1</v>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>What's the most useless talent you have?</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Just for Fun</t>
+        </is>
+      </c>
+      <c r="B133" t="n">
+        <v>1</v>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>If you had to eat one meal for the rest of your life, what is it?</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Just for Fun</t>
+        </is>
+      </c>
+      <c r="B134" t="n">
+        <v>1</v>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>What's your most controversial (totally non-serious) opinion?</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Just for Fun</t>
+        </is>
+      </c>
+      <c r="B135" t="n">
+        <v>1</v>
+      </c>
+      <c r="C135" t="inlineStr">
         <is>
           <t>If you were a UW–Madison building, which would you be and why?</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Just for Fun</t>
+        </is>
+      </c>
+      <c r="B136" t="n">
+        <v>1</v>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>What's a hill you'll die on that absolutely does not matter?</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Just for Fun</t>
+        </is>
+      </c>
+      <c r="B137" t="n">
+        <v>1</v>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>What fictional world would you most want to live in?</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Just for Fun</t>
+        </is>
+      </c>
+      <c r="B138" t="n">
+        <v>1</v>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Dinner with any three people, living or not — who's at the table?</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Just for Fun</t>
+        </is>
+      </c>
+      <c r="B139" t="n">
+        <v>1</v>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>What's the weirdest food combo you genuinely enjoy?</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Just for Fun</t>
+        </is>
+      </c>
+      <c r="B140" t="n">
+        <v>1</v>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>You get one superpower but it's mildly inconvenient — what is it?</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Just for Fun</t>
+        </is>
+      </c>
+      <c r="B141" t="n">
+        <v>1</v>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>What's your go-to hype song before something big?</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Just for Fun</t>
+        </is>
+      </c>
+      <c r="B142" t="n">
+        <v>1</v>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>What's the best purchase you've made under $20?</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Just for Fun</t>
+        </is>
+      </c>
+      <c r="B143" t="n">
+        <v>1</v>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>If your life had an entrance theme song, what plays when you walk in?</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Just for Fun</t>
+        </is>
+      </c>
+      <c r="B144" t="n">
+        <v>1</v>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>What's a snack or food take you'll defend to the end?</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Just for Fun</t>
+        </is>
+      </c>
+      <c r="B145" t="n">
+        <v>1</v>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>If you had unlimited money for one day, what's the first thing you buy?</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Just for Fun</t>
+        </is>
+      </c>
+      <c r="B146" t="n">
+        <v>1</v>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>What's your toxic trait as a group-project partner?</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Just for Fun</t>
+        </is>
+      </c>
+      <c r="B147" t="n">
+        <v>1</v>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>What's the pettiest reason you've stopped watching a show?</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>This or That</t>
+        </is>
+      </c>
+      <c r="B148" t="n">
+        <v>1</v>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Deep dish or thin crust?</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>This or That</t>
+        </is>
+      </c>
+      <c r="B149" t="n">
+        <v>1</v>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Text or call?</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>This or That</t>
+        </is>
+      </c>
+      <c r="B150" t="n">
+        <v>1</v>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Mountains or ocean?</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>This or That</t>
+        </is>
+      </c>
+      <c r="B151" t="n">
+        <v>1</v>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Sweet or salty?</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>This or That</t>
+        </is>
+      </c>
+      <c r="B152" t="n">
+        <v>1</v>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Window or aisle seat?</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>This or That</t>
+        </is>
+      </c>
+      <c r="B153" t="n">
+        <v>1</v>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Beach day or mountain day?</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>This or That</t>
+        </is>
+      </c>
+      <c r="B154" t="n">
+        <v>1</v>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Summer or winter?</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>This or That</t>
+        </is>
+      </c>
+      <c r="B155" t="n">
+        <v>1</v>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Books or movies?</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>This or That</t>
+        </is>
+      </c>
+      <c r="B156" t="n">
+        <v>1</v>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Cats or dogs?</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>This or That</t>
+        </is>
+      </c>
+      <c r="B157" t="n">
+        <v>1</v>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Big party or small hangout?</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>This or That</t>
+        </is>
+      </c>
+      <c r="B158" t="n">
+        <v>1</v>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Sneakers or slides?</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>This or That</t>
+        </is>
+      </c>
+      <c r="B159" t="n">
+        <v>1</v>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Group chat or one-on-one?</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>This or That</t>
+        </is>
+      </c>
+      <c r="B160" t="n">
+        <v>1</v>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Save it or spend it?</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>This or That</t>
+        </is>
+      </c>
+      <c r="B161" t="n">
+        <v>1</v>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Spicy or mild?</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>This or That</t>
+        </is>
+      </c>
+      <c r="B162" t="n">
+        <v>1</v>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Road trip or flight?</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>This or That</t>
+        </is>
+      </c>
+      <c r="B163" t="n">
+        <v>1</v>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Sunrise or sunset?</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>This or That</t>
+        </is>
+      </c>
+      <c r="B164" t="n">
+        <v>1</v>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Study in silence or study with music?</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>This or That</t>
+        </is>
+      </c>
+      <c r="B165" t="n">
+        <v>1</v>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Handwritten notes or laptop notes?</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>This or That</t>
+        </is>
+      </c>
+      <c r="B166" t="n">
+        <v>1</v>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Reply instantly or leave on read?</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>This or That</t>
+        </is>
+      </c>
+      <c r="B167" t="n">
+        <v>1</v>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Throwback hits or new releases?</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>This or That</t>
+        </is>
+      </c>
+      <c r="B168" t="n">
+        <v>1</v>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Big city or small town?</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>This or That</t>
+        </is>
+      </c>
+      <c r="B169" t="n">
+        <v>1</v>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Pancakes or waffles?</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>This or That</t>
+        </is>
+      </c>
+      <c r="B170" t="n">
+        <v>1</v>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Aux cord or let someone else DJ?</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>This or That</t>
+        </is>
+      </c>
+      <c r="B171" t="n">
+        <v>1</v>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Breakfast for dinner: yes or no?</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="B172" t="n">
+        <v>2</v>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Who's someone who feels like family, related or not?</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="B173" t="n">
+        <v>2</v>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>What's a tradition you grew up with that you'd want to keep someday?</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="B174" t="n">
+        <v>2</v>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>What's a lesson about life you picked up from the people who raised you?</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="B175" t="n">
+        <v>2</v>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Who did you go to for advice growing up, and about what?</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="B176" t="n">
+        <v>2</v>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>What's a meal or dish that tastes like home?</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="B177" t="n">
+        <v>3</v>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>In what ways are you like the people who raised you?</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="B178" t="n">
+        <v>3</v>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>What's something that felt totally normal growing up that you now realize was kind of special?</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="B179" t="n">
+        <v>2</v>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Who in your family are you most proud to be connected to?</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="B180" t="n">
+        <v>2</v>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>What's a story your family always tells about you?</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="B181" t="n">
+        <v>2</v>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>What's a piece of advice from a family member that stuck with you?</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="B182" t="n">
+        <v>3</v>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Who's a relative or elder whose story you wish you knew more about?</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="B183" t="n">
+        <v>3</v>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>What's a way your family shows love, even without saying it?</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="B184" t="n">
+        <v>2</v>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>What tradition or recipe do you hope to pass on someday?</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="B185" t="n">
+        <v>2</v>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>If you could thank one person who helped raise you, who is it and for what?</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>What Grounds You</t>
+        </is>
+      </c>
+      <c r="B186" t="n">
+        <v>2</v>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>What keeps you grounded when things get stressful?</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>What Grounds You</t>
+        </is>
+      </c>
+      <c r="B187" t="n">
+        <v>2</v>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>What's a belief or practice that matters to you?</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>What Grounds You</t>
+        </is>
+      </c>
+      <c r="B188" t="n">
+        <v>2</v>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Where do you feel most at peace?</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>What Grounds You</t>
+        </is>
+      </c>
+      <c r="B189" t="n">
+        <v>2</v>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>What's a small ritual or routine that centers you?</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>What Grounds You</t>
+        </is>
+      </c>
+      <c r="B190" t="n">
+        <v>3</v>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>What does faith — in anything — mean to you?</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>What Grounds You</t>
+        </is>
+      </c>
+      <c r="B191" t="n">
+        <v>3</v>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Who or what do you turn to when you need strength?</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>What Grounds You</t>
+        </is>
+      </c>
+      <c r="B192" t="n">
+        <v>4</v>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>What gives your life a sense of meaning right now?</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>What Grounds You</t>
+        </is>
+      </c>
+      <c r="B193" t="n">
+        <v>2</v>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>What do you do to reset when you're overwhelmed?</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>What Grounds You</t>
+        </is>
+      </c>
+      <c r="B194" t="n">
+        <v>2</v>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>What's a saying, prayer, or mantra that gives you strength?</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>What Grounds You</t>
+        </is>
+      </c>
+      <c r="B195" t="n">
+        <v>3</v>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>What's something bigger than yourself that you feel connected to?</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>What Grounds You</t>
+        </is>
+      </c>
+      <c r="B196" t="n">
+        <v>3</v>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>How do you want to grow, spiritually or personally, in college?</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>What Grounds You</t>
+        </is>
+      </c>
+      <c r="B197" t="n">
+        <v>2</v>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>What's a value or practice from home you want to hold onto here?</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>Your Posse</t>
+        </is>
+      </c>
+      <c r="B198" t="n">
+        <v>2</v>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>What are you most excited about starting this journey with a Posse?</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>Your Posse</t>
+        </is>
+      </c>
+      <c r="B199" t="n">
+        <v>2</v>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>What's something you're nervous about as you start college with a new crew?</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>Your Posse</t>
+        </is>
+      </c>
+      <c r="B200" t="n">
+        <v>3</v>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>What does real support from a friend look like to you?</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>Your Posse</t>
+        </is>
+      </c>
+      <c r="B201" t="n">
+        <v>3</v>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>How do you want to show up for your Posse this year?</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>Your Posse</t>
+        </is>
+      </c>
+      <c r="B202" t="n">
+        <v>3</v>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>What do you hope your Posse becomes to each other by senior year?</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>Your Posse</t>
+        </is>
+      </c>
+      <c r="B203" t="n">
+        <v>2</v>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>What's a strength you bring to a group?</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>Your Posse</t>
+        </is>
+      </c>
+      <c r="B204" t="n">
+        <v>4</v>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>What do you need from the people around you to feel like you belong?</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>Your Posse</t>
+        </is>
+      </c>
+      <c r="B205" t="n">
+        <v>2</v>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>What does being part of a Posse mean to you?</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>Your Posse</t>
+        </is>
+      </c>
+      <c r="B206" t="n">
+        <v>4</v>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>How can this group have your back when things get hard?</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>Your Posse</t>
+        </is>
+      </c>
+      <c r="B207" t="n">
+        <v>3</v>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>What's one way you want to grow with this group over the next four years?</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>Your Posse</t>
+        </is>
+      </c>
+      <c r="B208" t="n">
+        <v>4</v>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>What do you hope your Posse remembers about you?</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>Your Posse</t>
+        </is>
+      </c>
+      <c r="B209" t="n">
+        <v>2</v>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>What's something you'd love for this group to do together?</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>Your Posse</t>
+        </is>
+      </c>
+      <c r="B210" t="n">
+        <v>2</v>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>What kind of friend are you hoping to be here?</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>Your Posse</t>
+        </is>
+      </c>
+      <c r="B211" t="n">
+        <v>3</v>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>When has a group made you feel like you truly belonged?</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>Your Posse</t>
+        </is>
+      </c>
+      <c r="B212" t="n">
+        <v>4</v>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>What's something you hope you can all be honest with each other about?</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>Your Posse</t>
+        </is>
+      </c>
+      <c r="B213" t="n">
+        <v>3</v>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>What would make this Posse feel like a home away from home?</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>Your Posse</t>
+        </is>
+      </c>
+      <c r="B214" t="n">
+        <v>2</v>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>How do you hope you'll all celebrate each other's wins?</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>Your Posse</t>
+        </is>
+      </c>
+      <c r="B215" t="n">
+        <v>3</v>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>What's a promise you'd want everyone in this Posse to make to each other?</t>
         </is>
       </c>
     </row>

</xml_diff>